<commit_message>
Cover Parth optimization gaps in v10 core
</commit_message>
<xml_diff>
--- a/docs/subagent_query_bank-v1.xlsx
+++ b/docs/subagent_query_bank-v1.xlsx
@@ -557,8 +557,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -631,17 +631,175 @@
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>For LDPE/EVOH/PET at 100 C, generate the top 5 dynamic-programming separation sequences and report the solvent, operating temperature, and selectivity for each step.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>live-tested</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>DP separation sequence ranking for three-polymer feedstock</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>separation-engineer</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>plan_sequential_separation or plan_multiple_separation_schemes</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>polymers=LDPE,EVOH,PET; operating_temperature_c=100; top_k=5</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>ranked separation sequences; per-step solvent, temperature, selectivity</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Uses separation planning tools, not HSP/statistics; reports actual step temperatures and candidate route ranking.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/01_01_separation_engineer_r2</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Rank solvents for selectively dissolving LDPE over PET at 120 C and report the top 5 candidates with selectivity and atmospheric-pressure caveats.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>live-tested</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>pairwise selective-solubility solvent ranking with boiling-point caveats</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>separation-engineer</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>rank_solvents_for_separation</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>target_polymer=LDPE; comparison_polymer=PET; temperature_c=120; top_k=5</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ranked solvent table; selectivity metrics; atmospheric feasibility notes</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Does not route to statistics-ml unless HSP/RED is explicitly requested; avoids above-BP recommendations.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/02_01_separation_engineer_r3</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Find optimal separation conditions below 160 C for dissolving EVOH while leaving LDPE and PET behind; report the best solvent, temperature, selectivity, and model caveats.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>live-tested</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>temperature-search selective dissolution for EVOH target</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>separation-engineer</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>find_optimal_separation_conditions or analyze_selective_solubility_enhanced</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>target_polymer=EVOH; other_polymers=LDPE,PET; max_temperature_c=160</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>best solvent-temperature condition; selectivity; caveats</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Treats 160 C as upper bound, not fixed temperature; clearly labels fitted-model caveats.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/03_01_separation_engineer_r4</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K2"/>
@@ -694,8 +852,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -1326,6 +1484,63 @@
       <c r="K11" s="3" t="inlineStr">
         <is>
           <t>Heavier future regression. Use after fixed-slice harness remains stable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Run a cost-vs-circularity Pareto landscape for a mixed plastic feedstock of 8000 tonnes/year composed of 25% PP, 25% PS, 25% PVC, and 25% PC under scenario A with 12 points, requiring at least 1 STRAP wash and allowing up to 2 washes. Use these optimizer-supported shortlisted solvent candidates: PP: Toluene and Cyclohexane; PS: Toluene and N,N-Dimethylformamide; PVC: N,N-Dimethylformamide and Dimethyl sulfoxide; PC: Toluene and N,N-Dimethylformamide. Constrain the Pareto frontier to the one-wash PVC-Dimethyl sulfoxide residual route, but keep the candidate-pool landscape points visible. Plot the resulting Pareto landscape, title it "PP/PS/PVC/PC Pareto Landscape with Residual Polymer Routing", and save the PNG to "/home/aaltamimi2/langchain-STRAP-v10-core/case-studies/case-2-validation/Pareto-4-polymer/optimization_pareto_circularity_pp25_ps25_pvc25_pc25_residuals_20260427.png". Report the frontier points and saved path.</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>validated</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>4-polymer cost-vs-circularity Pareto landscape with residual polymer routing</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>typed runtime selected optimization -&gt; visualization-specialist</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>run_waste_management_pareto; plot_optimization_pareto_front</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>feed=8000 tpy; composition PP/PS/PVC/PC=25/25/25/25; scenario=A; n_points=12; x_metric=total_cost; y_metric=circularity; min_washes=1; max_washes=2; shortlisted candidates PP=Toluene/Cyclohexane, PS=Toluene/N,N-Dimethylformamide, PVC=N,N-Dimethylformamide/Dimethyl sulfoxide, PC=Toluene/N,N-Dimethylformamide; frontier constrained to one-wash PVC-DMSO residual route; output PNG path</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>optimization_pareto_front payload; optimization_pareto_landscape payload with candidate-pool landscape points; optimization_pareto_plot PNG</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Actual dissolve CLI with DISSOLVE_TYPED_PLANNER=enforce_selected uses typed_runtime, not direct solubility fast path; frontier has 2 points; landscape has 32 candidate points; PNG is 3415x1361 and saved under v10-core case-2-validation.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/case-studies/case-2-validation/Pareto-4-polymer/optimization_pareto_circularity_pp25_ps25_pvc25_pc25_residuals_20260427.png</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Validated 2026-04-27 through python -m strap.claude_sdk_harness.cli --mode auto --no-persist; transcript: /home/aaltamimi2/langchain-STRAP-v10-core/case-studies/case-2-validation/Pareto-4-polymer/dissolve_cli_validation_transcript.txt. Regression fixed: selected Pareto query must bypass direct solubility fast path.</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1606,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -2084,8 +2299,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2158,17 +2373,175 @@
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Run BioSTEAM TEA/LCA for LDPE with Cyclohexane under energy case C2 and report MSP, TCI, AOC, GWP, and the boiling-point margin.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>live-tested</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>single BioSTEAM TEA/LCA simulation with physical feasibility margin</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>biosteam-analyst</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>run_biosteam_simulation</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>target_plastic=LDPE; solvent=Cyclohexane; energy_case=C2</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>tea.lca metrics: MSP, TCI, AOC, GWP; process-condition caveats</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Reports all four required BioSTEAM metrics and does not substitute optimization output.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/04_03_biosteam_analyst_r2</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Compare BioSTEAM TEA/LCA for PET using Toluene versus Dimethyl sulfoxide under energy case C1; report MSP, TCI, AOC, GWP, failed scenarios, and the lower-MSP solvent.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>live-tested</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>BioSTEAM batch solvent comparison with failure reporting</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>biosteam-analyst</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>run_biosteam_batch</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>target_plastic=PET; solvents=Toluene,Dimethyl sulfoxide; energy_case=C1</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>batch TEA/LCA comparison; success/failure records; best solvent by MSP</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Continues if one solvent fails; includes MSP, TCI, AOC, and GWP for retained scenarios.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/05_03_biosteam_analyst_r3</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Run a BioSTEAM multi-polymer recovery case under energy case C3 for PE dissolved with Toluene followed by EVOH dissolved with Ethylene glycol; report blended MSP, combined TCI, weighted GWP, and per-step conditions.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>live-tested</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>multi-polymer sequential BioSTEAM recovery metrics</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>biosteam-analyst</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>run_biosteam_multi_polymer</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>polymers_json=[PE/Toluene,EVOH/Ethylene glycol]; energy_case=C3</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>multi-polymer TEA/LCA result; blended MSP; combined TCI; weighted GWP</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Runs multi-polymer tool rather than separate prose-only estimates; reports per-step caveats.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/06_03_biosteam_analyst_r4</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K2"/>
@@ -2221,8 +2594,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2295,17 +2668,161 @@
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Search Google Scholar for solvent-based recycling of multilayer LDPE/EVOH/PET packaging films and summarize the top 5 relevant papers with year, DOI if available, and relevance to selective dissolution.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>pending-live</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>literature search for multilayer selective-dissolution recycling</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>scholar-researcher</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>search_google_scholar</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>topic=solvent-based recycling multilayer LDPE EVOH PET packaging selective dissolution</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>paper list with citations/years/DOIs when available</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Uses scholar search tooling and cites source metadata rather than unsupported claims.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Run after process/visualization domains because external search can be slow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Search arXiv for machine-learning models for polymer solubility or Hansen parameters in solvent-based plastic recycling; summarize methods, datasets, and data limitations.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending-live</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>arXiv literature search for polymer-solubility ML/HSP models</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>scholar-researcher</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>search_arxiv</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>topic=machine learning polymer solubility Hansen parameters solvent recycling</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>paper summary with methods/datasets/limitations</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Uses arXiv/scholar tooling; distinguishes papers from model-internal claims.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Run after process/visualization domains because external search can be slow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Search Web of Science for recent TEA/LCA studies of solvent-based plastic recycling and compare their main cost and emissions conclusions.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pending-live</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TEA/LCA literature search and comparison</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>scholar-researcher</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>search_web_of_science</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>topic=TEA LCA solvent-based plastic recycling cost emissions</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>recent paper comparison with cost/emissions conclusions</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Uses literature-search tool; clearly reports API/data limitations if search unavailable.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Run after process/visualization domains because external search can be slow.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K2"/>
@@ -2358,8 +2875,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2432,17 +2949,161 @@
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Search Google Patents for solvent-based recycling of multilayer polyethylene/EVOH/PET packaging and summarize the most relevant patent families, assignees, and claimed solvent systems.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>pending-live</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>patent search for multilayer packaging solvent recycling</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>patent-researcher</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>search_google_patents</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>topic=solvent-based recycling multilayer polyethylene EVOH PET packaging</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>patent family/assignee/claim summary</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Uses patent-search tooling; avoids conflating papers with patents.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Run after process/visualization domains because external search can be slow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Search polymer patents for selective dissolution of polyolefins using xylene, toluene, or dodecane and report assignees, target polymers, and claimed temperature ranges.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending-live</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>polyolefin selective-dissolution patent search</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>patent-researcher</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>search_polymer_patents</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>topic=polyolefin selective dissolution xylene toluene dodecane temperature</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>patent list with assignees, polymers, temperature claims</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Uses patent tools and reports temperature ranges only when present in source metadata.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Run after process/visualization domains because external search can be slow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Search patents related to removing phthalates or PFAS contaminants from recycled polymers using solvent extraction; summarize the strongest claims and polymer targets.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pending-live</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>contaminant-removal patent search</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>patent-researcher</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>search_google_patents or search_patentsview</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>topic=phthalate PFAS contaminant removal recycled polymer solvent extraction patent</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>patent summary with claims and target polymers</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Uses patent source metadata; reports unavailable fields as gaps.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Run after process/visualization domains because external search can be slow.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K2"/>
@@ -2495,8 +3156,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2569,17 +3230,161 @@
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Ask the literature RAG what the local corpus says about STRAP solvent selection for PE/EVOH/PET multilayer separations, and cite the retrieved chunks.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>pending-live</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>RAG answer over local corpus for solvent selection</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>rag-analyst</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>ask_literature or search_literature_rag</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>question=STRAP solvent selection PE EVOH PET multilayer separation</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>RAG answer with cited retrieved chunks</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Uses local RAG retrieval and clearly says if index is empty/unavailable.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Run last because RAG state may depend on local index contents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Search the literature RAG for BioSTEAM TEA/LCA assumptions used in STRAP recycling and summarize the cited source chunks for MSP, TCI, AOC, and GWP.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending-live</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>RAG retrieval for BioSTEAM TEA/LCA assumptions</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>rag-analyst</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>search_literature_rag</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>query=BioSTEAM STRAP TEA LCA MSP TCI AOC GWP assumptions</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>retrieved chunks and metric-assumption summary</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Does not fabricate source chunks; distinguishes no-hit retrieval from domain answer.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Run last because RAG state may depend on local index contents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Get the RAG status, then answer whether local documents mention contaminant-aware solvent selection or PFAS/phthalate removal in recycled polymers.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pending-live</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>RAG status plus contaminant-aware retrieval query</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>rag-analyst</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>get_rag_status and ask_literature</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>question=contaminant-aware solvent selection PFAS phthalate removal recycled polymers</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>RAG status plus cited answer or no-hit diagnostic</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Reports index status before answering; no unsupported citations.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Run last because RAG state may depend on local index contents.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K2"/>
@@ -2632,8 +3437,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2706,17 +3511,175 @@
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Plot the solubility of LDPE, PET, and EVOH in dodecane and o-xylene from 25 C to 160 C with a normalized 0-100% y-axis. Save the PNG to "/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/visualization/solubility".</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>live-tested</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>multi-polymer multi-solvent solubility plot with normalized y-axis</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>visualization-specialist</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>plot_solubility_vs_temperature</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>polymers=LDPE,PET,EVOH; solvents=dodecane,o-xylene; temp_range=25-160; output_dir</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>PNG solubility plot path; normalized 0-100% y-axis</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Preserves all requested polymers/solvents; does not narrow to a prior context pair.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/07_07_visualization_specialist_r2</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Generate a dynamic-programming separation state map for LDPE/EVOH/PET at 100 C and save it to "/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/visualization/dp_state_map". Only include separation/selectivity visuals, not cost or greenness plots.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>live-tested</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>DP state-map visualization without objective overlays</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>visualization-specialist</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>plot_dynamic_programming_separation_options</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>polymers=LDPE,EVOH,PET; temperature_c=100; output_dir</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>separation sequence PNGs and DP state map artifact</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Uses DP separation plotting, not solubility plotting; avoids cost/greenness objective paths.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/08_07_visualization_specialist_r3</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Create a simple separation tree plot for LDPE/EVOH/PET at 100 C, including solvent and temperature labels, and save it to "/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/visualization/separation_tree".</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>live-tested</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>simple separation tree/flowchart visualization</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>visualization-specialist</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>create_separation_tree_plot</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>polymers=LDPE,EVOH,PET; temperature_c=100; output_dir</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>separation tree PNG path</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Uses tree/flowchart visualization, not full DP objective plotting unless explicitly needed.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/09_07_visualization_specialist_r4</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K2"/>
@@ -2770,7 +3733,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -3463,8 +4426,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -3537,17 +4500,161 @@
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Screen leaching-mode removal of di-n-butyl phthalate (DBP) from PET using acetone, ethyl acetate, and cyclohexane up to 55 C while keeping PET intact.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>pending-live</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>phthalate leaching screen with polymer-intact criterion</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>contaminant-removal-analyst</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>screen_contaminant_leaching</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>target_polymer=PET; contaminant=di-n-butyl phthalate (DBP); solvents=acetone,ethyl acetate,cyclohexane; max_temperature_c=55</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>contaminant leaching candidate solvent table; recommended solvents</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Uses contaminant-removal data; states unsupported solvents/contaminants explicitly.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Gemini Flash Lite live harness candidate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Compare leaching versus STRAP temperature-swing contaminant removal for Perfluorooctanoic Acid from LDPE using toluene, cyclohexane, and dodecane up to 120 C.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending-live</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mode comparison for PFAS removal from LDPE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>contaminant-removal-analyst</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>compare_contaminant_removal_modes</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>target_polymer=LDPE; contaminant=Perfluorooctanoic Acid; solvents=toluene,cyclohexane,dodecane; max_temperature_c=120</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>side-by-side leaching vs STRAP contaminant-removal result</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Does not invent contaminant partition data; calls out atmospheric constraints near solvent BP.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Gemini Flash Lite live harness candidate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>For PET contaminated with DEHP and BBP, screen STRAP contaminant removal by temperature-swing precipitation using dodecane and o-xylene below 140 C.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pending-live</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>multi-contaminant STRAP temperature-swing screen</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>contaminant-removal-analyst</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>screen_contaminant_strap_removal</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>target_polymer=PET; contaminants=DEHP,BBP; solvents=dodecane,o-xylene; max_temperature_c=140</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>STRAP contaminant-removal candidate table and caveats</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Uses temperature-swing STRAP tool; reports if no solvent passes blocking criteria.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Gemini Flash Lite live harness candidate.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K2"/>

</xml_diff>

<commit_message>
Add latest contaminant query validation results
</commit_message>
<xml_diff>
--- a/docs/subagent_query_bank-v1.xlsx
+++ b/docs/subagent_query_bank-v1.xlsx
@@ -4507,7 +4507,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>pending-live</t>
+          <t>live-tested</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -4545,10 +4545,14 @@
           <t>Uses contaminant-removal data; states unsupported solvents/contaminants explicitly.</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/10_09_contaminant_removal_r2</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Gemini Flash Lite live harness candidate.</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
         </is>
       </c>
     </row>
@@ -4560,7 +4564,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pending-live</t>
+          <t>live-tested</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4598,9 +4602,14 @@
           <t>Does not invent contaminant partition data; calls out atmospheric constraints near solvent BP.</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/11_09_contaminant_removal_r3</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Gemini Flash Lite live harness candidate.</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
         </is>
       </c>
     </row>
@@ -4612,7 +4621,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>pending-live</t>
+          <t>live-tested</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4650,9 +4659,14 @@
           <t>Uses temperature-swing STRAP tool; reports if no solvent passes blocking criteria.</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/12_09_contaminant_removal_r4</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Gemini Flash Lite live harness candidate.</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add research query bank validation results
</commit_message>
<xml_diff>
--- a/docs/subagent_query_bank-v1.xlsx
+++ b/docs/subagent_query_bank-v1.xlsx
@@ -558,7 +558,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>live-tested</t>
+          <t>live-tested-needs-review</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; semantic issue: query specified 100 C, but response recommended 137.3 C and 160.0 C step temperatures. Needs fixed-temperature routing/wording review. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/01_01_separation_engineer_r2</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -1606,7 +1606,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -2300,7 +2300,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>live-tested</t>
+          <t>live-tested-needs-fix</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; typed runtime succeeded but user-facing response only reported plan/bundle, not requested MSP/TCI/AOC/GWP/boiling margin. Metrics exist in diagnostic artifacts. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/04_03_biosteam_analyst_r2</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>live-tested</t>
+          <t>live-tested-needs-fix</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; typed compiler captured both solvents but executed run_biosteam_simulation for Toluene only, not run_biosteam_batch; response did not compare DMSO or lower-MSP solvent. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/05_03_biosteam_analyst_r3</t>
         </is>
       </c>
     </row>
@@ -2494,7 +2494,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>live-tested</t>
+          <t>live-tested-needs-fix</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Gemini Flash Lite CLI live run 2026-04-27; rc=0; timeout=False</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; typed compiler executed single PE/Toluene run instead of run_biosteam_multi_polymer for PE then EVOH; blended MSP/combined TCI/weighted GWP not reported. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/priority/06_03_biosteam_analyst_r4</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2595,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2675,7 +2675,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>pending-live</t>
+          <t>live-tested-needs-review</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2713,10 +2713,14 @@
           <t>Uses scholar search tooling and cites source metadata rather than unsupported claims.</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/01_04_scholar_researcher_r2</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Run after process/visualization domains because external search can be slow.</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; response returned paper table after ~151s but citations/source metadata need manual review before marking validated. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/01_04_scholar_researcher_r2</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2732,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pending-live</t>
+          <t>live-failed</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2766,9 +2770,14 @@
           <t>Uses arXiv/scholar tooling; distinguishes papers from model-internal claims.</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/02_04_scholar_researcher_r3</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Run after process/visualization domains because external search can be slow.</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; typed runtime intercepted as selected HSP screen and failed compile due missing concrete polymer/solvent, instead of routing to scholar/arXiv search. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/02_04_scholar_researcher_r3</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2789,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>pending-live</t>
+          <t>live-failed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2818,9 +2827,14 @@
           <t>Uses literature-search tool; clearly reports API/data limitations if search unavailable.</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/03_04_scholar_researcher_r4</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Run after process/visualization domains because external search can be slow.</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; typed runtime intercepted as selected BioSTEAM/TEA-LCA and returned clarification_required instead of routing to Web of Science scholar search. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/03_04_scholar_researcher_r4</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2890,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2956,7 +2970,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>pending-live</t>
+          <t>live-failed</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2994,10 +3008,14 @@
           <t>Uses patent-search tooling; avoids conflating papers with patents.</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/04_05_patent_researcher_r2</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Run after process/visualization domains because external search can be slow.</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; patent search route reached patent agent but live patent retrieval failed because external patent API keys/config were unavailable. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/04_05_patent_researcher_r2</t>
         </is>
       </c>
     </row>
@@ -3009,7 +3027,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pending-live</t>
+          <t>live-failed</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3047,9 +3065,14 @@
           <t>Uses patent tools and reports temperature ranges only when present in source metadata.</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/05_05_patent_researcher_r3</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Run after process/visualization domains because external search can be slow.</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; patent search route reached patent agent but SerpAPI/PatentsView keys were unavailable, so no patent data was retrieved. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/05_05_patent_researcher_r3</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3084,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>pending-live</t>
+          <t>live-failed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3099,9 +3122,14 @@
           <t>Uses patent source metadata; reports unavailable fields as gaps.</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/06_05_patent_researcher_r4</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Run after process/visualization domains because external search can be slow.</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; patent search did not retrieve live patent data and stderr included unawaited get_rag_status coroutine plus RecursionError while formatting warning. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/06_05_patent_researcher_r4</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3185,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -3237,7 +3265,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>pending-live</t>
+          <t>live-failed</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -3275,10 +3303,14 @@
           <t>Uses local RAG retrieval and clearly says if index is empty/unavailable.</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/07_06_rag_analyst_r2</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Run last because RAG state may depend on local index contents.</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; query asked literature RAG over local corpus, but response routed to available-solvents listing instead of RAG retrieval/chunk citations. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/07_06_rag_analyst_r2</t>
         </is>
       </c>
     </row>
@@ -3290,7 +3322,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pending-live</t>
+          <t>live-failed</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3328,9 +3360,14 @@
           <t>Does not fabricate source chunks; distinguishes no-hit retrieval from domain answer.</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/08_06_rag_analyst_r3</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Run last because RAG state may depend on local index contents.</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; typed runtime intercepted as selected BioSTEAM/TEA-LCA and returned clarification_required instead of routing to RAG retrieval. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/08_06_rag_analyst_r3</t>
         </is>
       </c>
     </row>
@@ -3342,7 +3379,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>pending-live</t>
+          <t>live-tested-needs-review</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3380,9 +3417,14 @@
           <t>Reports index status before answering; no unsupported citations.</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>/home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/09_06_rag_analyst_r4</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Run last because RAG state may depend on local index contents.</t>
+          <t>Gemini Flash Lite CLI live run 2026-04-27; response answered from broad system/document context but did not provide explicit retrieved chunk citations as requested. Transcript: /home/aaltamimi2/langchain-STRAP-v10-core/architecture/test_results/query_bank_live_gemini_20260427/research_last/09_06_rag_analyst_r4</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3480,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -3733,7 +3775,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -4427,7 +4469,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>

</xml_diff>